<commit_message>
fix: finalize A group image translation pipeline
</commit_message>
<xml_diff>
--- a/collaboration/groups/A_image_translation/deliverables/extracted_20260717_update/manifests/translation_manifest_reviewed.xlsx
+++ b/collaboration/groups/A_image_translation/deliverables/extracted_20260717_update/manifests/translation_manifest_reviewed.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reviewed translations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="reviewed translations" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'reviewed translations'!$A$1:$L$72</definedName>
@@ -549,12 +549,12 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Harmony between humanity and nature; the spirit of Confucianism, Daoism, and Chan</t>
+          <t>Harmony between humanity and nature; Confucian, Daoist, and Chan wisdom</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -603,12 +603,12 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Cultivate virtue; follow the way of nature</t>
+          <t>Cultivate the self and virtue; follow nature's way</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -657,12 +657,12 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Confucianism cultivates virtue in society; Daoism embraces natural freedom</t>
+          <t>Confucians engage with society and cultivate virtue; Daoists live freely and at ease</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -711,12 +711,12 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -765,12 +765,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -819,12 +819,12 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -873,12 +873,12 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Poetry holds landscapes; writing bears witness to the ages</t>
+          <t>Poetry and rhapsody embrace the land; writing bears witness to the ages</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -927,12 +927,12 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -981,12 +981,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The Chinese spirit in poetry, lyrics, drama, and prose</t>
+          <t>The Chinese spirit in poetry, lyric verse, songs, and rhapsodies</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1068,7 +1068,7 @@
       <c r="D12" s="2" t="inlineStr">
         <is>
           <t>The Book of Songs:
-collecting folk ballads</t>
+gathering folk songs</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1123,20 +1123,20 @@
       <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Qu Yuan chants
-by the river</t>
+by the waterside</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>425</v>
+        <v>340</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>540</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>515</v>
+        <v>550</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1145,12 +1145,12 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1255,12 +1255,12 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1288,7 +1288,7 @@
       <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Cao Xueqin
-writes</t>
+writes a novel</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>The grandeur of the Tang; the elegance of the Song</t>
+          <t>High Tang grandeur; Northern and Southern Song elegance</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -1364,12 +1364,12 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1418,12 +1418,12 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -1472,12 +1472,12 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>The brush summons clouds; ink shapes mountains and waters</t>
+          <t>A brushstroke conjures clouds; ink forms mountains and waters</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1580,12 +1580,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Gardens encompass a world; bricks and tiles reveal poetry</t>
+          <t>Gardens contain worlds; bricks and tiles reveal poetry</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Mortise and tenon interlock; bricks and tiles become poetry</t>
+          <t>Mortise-and-tenon joints interlock; bricks and tiles become poetry</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
@@ -1688,12 +1688,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -1742,12 +1742,12 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -1796,12 +1796,12 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -1850,12 +1850,12 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Each region, its own landscape and dwellings</t>
+          <t>Each place has its own landscape and dwellings</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -1904,12 +1904,12 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -1958,12 +1958,12 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2012,12 +2012,12 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2066,12 +2066,12 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2121,12 +2121,12 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2229,12 +2229,12 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Craftsmanship shapes each object; artifacts carry civilization</t>
+          <t>Every object embodies craftsmanship; artifacts carry civilization</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -2283,12 +2283,12 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2337,12 +2337,12 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2391,12 +2391,12 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -2499,12 +2499,12 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Sericulture and silk weaving connected Eastern and Western civilizations</t>
+          <t>Sericulture and silk reeling linked Eastern and Western civilizations</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
@@ -2553,12 +2553,12 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -2607,12 +2607,12 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -2715,12 +2715,12 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>One stage, one story</t>
+          <t>Every stage tells a story</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
@@ -2769,12 +2769,12 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Over 300 opera traditions take root in local communities</t>
+          <t>More than 300 opera genres are rooted in local communities</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -2877,12 +2877,12 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -2931,12 +2931,12 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -2985,12 +2985,12 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -3039,12 +3039,12 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -3093,12 +3093,12 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Attire embodies ritual; ceremonial dress shines with distinction</t>
+          <t>Attire reflects ritual; ceremonial dress shines</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
@@ -3147,12 +3147,12 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -3201,12 +3201,12 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Different paths lead to the same end: a heart at peace</t>
+          <t>Different paths lead to the same destination; the heart seeks peace</t>
         </is>
       </c>
       <c r="E52" s="2" t="n">
@@ -3255,12 +3255,12 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -3301,12 +3301,12 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Harmony between humanity and nature; the spirit of Confucianism, Daoism, and Chan</t>
+          <t>Harmony between humanity and nature; Confucian, Daoist, and Chan wisdom</t>
         </is>
       </c>
       <c r="E54" s="2" t="n"/>
@@ -3347,12 +3347,12 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -3393,12 +3393,12 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Poetry holds landscapes; writing bears witness to the ages</t>
+          <t>Poetry and rhapsody embrace the land; writing bears witness to the ages</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>
@@ -3439,12 +3439,12 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -3485,12 +3485,12 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>The brush summons clouds; ink shapes mountains and waters</t>
+          <t>A brushstroke conjures clouds; ink forms mountains and waters</t>
         </is>
       </c>
       <c r="E58" s="2" t="n"/>
@@ -3531,12 +3531,12 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
@@ -3577,12 +3577,12 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Gardens encompass a world; bricks and tiles reveal poetry</t>
+          <t>Gardens contain worlds; bricks and tiles reveal poetry</t>
         </is>
       </c>
       <c r="E60" s="2" t="n"/>
@@ -3623,12 +3623,12 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -3669,12 +3669,12 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Craftsmanship shapes each object; artifacts carry civilization</t>
+          <t>Every object embodies craftsmanship; artifacts carry civilization</t>
         </is>
       </c>
       <c r="E62" s="2" t="n"/>
@@ -3715,12 +3715,12 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -3761,12 +3761,12 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
@@ -3807,12 +3807,12 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -3853,12 +3853,12 @@
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -3945,12 +3945,12 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
@@ -3991,12 +3991,12 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
@@ -4037,12 +4037,12 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Attire embodies ritual; ceremonial dress shines with distinction</t>
+          <t>Attire reflects ritual; ceremonial dress shines</t>
         </is>
       </c>
       <c r="E70" s="2" t="n"/>
@@ -4083,12 +4083,12 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Different paths lead to the same end: a heart at peace</t>
+          <t>Different paths lead to the same destination; the heart seeks peace</t>
         </is>
       </c>
       <c r="E72" s="2" t="n"/>
@@ -4175,12 +4175,12 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>Codex independent technical review</t>
+          <t>Codex independent technical and linguistic review</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">

</xml_diff>